<commit_message>
update flagging and comments for 4 new cruises
</commit_message>
<xml_diff>
--- a/data/input/DOC_20251024_AR88_AR92_AR95.xlsx
+++ b/data/input/DOC_20251024_AR88_AR92_AR95.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\sosiknas1.whoi.edu\Lab_data\LTER\DOC\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D17C38C-B65C-4DA5-BF2E-BDA60C3F01A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759E45ED-F258-43D4-98D2-5AAC0BA35F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2925" yWindow="2535" windowWidth="24945" windowHeight="13785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="158">
   <si>
     <t>L1</t>
   </si>
@@ -469,6 +480,36 @@
   </si>
   <si>
     <t>AR95_33</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial but duplciation excellent so keep as good</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial but duplciation excellent so keep as good. DUPLICATE</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial. DOC higher than same depth at adjacent stations which throws DOC:DTN ratio off - DOC likely bad but flag as questionable as of 6/3/26</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial - DOC substationally higher than any values in vicinity - clearly conaminated from particles making it into sample vial, DTN also substationally higher. Flag both as bad</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial - surf DOC higher than next 2 inshore stations - very likely inflated due to particle loading in vial from incorrect filtering. Nitrogen consistent with adjacent station surf valuse so flag as 3</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial.</t>
+  </si>
+  <si>
+    <t>Filter cartridge not asesmbled correctly - possible for particular to pass through into sample vial. - DOC appears lower than expected while DTN syncs up with other inner midshelf/inshore stations/ D:N ratio off compared to adjacent suf samples though</t>
+  </si>
+  <si>
+    <t>DOC lower than expected. Is it possible chlmax and surf vials were accidentally switched? Can't know for sure. Flag as 3</t>
+  </si>
+  <si>
+    <t>DOC significantly higher than adjancent stations and depths. Must be contaminated. Is it possible chlmax and surf vials were accidentally switched?  Nitrogen seems reasonable so flag as 3</t>
+  </si>
+  <si>
+    <t>DOC higher than expected for offshore surface waters. Could be real. Needs further investigation</t>
   </si>
 </sst>
 </file>
@@ -535,7 +576,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -545,6 +586,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -625,7 +672,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -658,40 +705,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -727,6 +741,39 @@
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1016,66 +1063,68 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="7" max="8" width="8.85546875"/>
+    <col min="7" max="7" width="8.85546875"/>
+    <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="12.42578125" customWidth="1"/>
-    <col min="11" max="11" width="25.42578125" style="21" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="70.140625" style="41" customWidth="1"/>
+    <col min="14" max="14" width="0" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="9.28515625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="I1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="J1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="K1" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="O1" s="27" t="s">
+      <c r="O1" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="27" t="s">
+      <c r="P1" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="Q1" s="28" t="s">
+      <c r="Q1" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="R1" s="28" t="s">
+      <c r="R1" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="S1" s="29" t="s">
+      <c r="S1" s="18" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1110,27 +1159,27 @@
       <c r="J2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="12"/>
-      <c r="L2" s="37">
-        <v>2</v>
-      </c>
-      <c r="M2" s="37">
-        <v>2</v>
-      </c>
-      <c r="O2" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P2" s="33" t="s">
+      <c r="K2" s="34"/>
+      <c r="L2" s="26">
+        <v>1</v>
+      </c>
+      <c r="M2" s="26">
+        <v>1</v>
+      </c>
+      <c r="O2" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P2" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="Q2" s="34">
+      <c r="Q2" s="23">
         <v>90.03159420289856</v>
       </c>
-      <c r="R2" s="38">
+      <c r="R2" s="27">
         <v>5.562066744140826</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -1161,27 +1210,29 @@
       <c r="J3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="13"/>
-      <c r="L3" s="37">
-        <v>2</v>
-      </c>
-      <c r="M3" s="37">
-        <v>2</v>
-      </c>
-      <c r="O3" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P3" s="33" t="s">
+      <c r="K3" s="35" t="s">
+        <v>153</v>
+      </c>
+      <c r="L3" s="26">
+        <v>3</v>
+      </c>
+      <c r="M3" s="26">
+        <v>3</v>
+      </c>
+      <c r="O3" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P3" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="Q3" s="34">
+      <c r="Q3" s="23">
         <v>73.591014492753615</v>
       </c>
-      <c r="R3" s="38">
+      <c r="R3" s="27">
         <v>4.7767334108074921</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
@@ -1212,23 +1263,25 @@
       <c r="J4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="13"/>
-      <c r="L4" s="37">
-        <v>2</v>
-      </c>
-      <c r="M4" s="37">
-        <v>2</v>
-      </c>
-      <c r="O4" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P4" s="33" t="s">
+      <c r="K4" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="L4" s="26">
+        <v>3</v>
+      </c>
+      <c r="M4" s="26">
+        <v>3</v>
+      </c>
+      <c r="O4" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P4" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="Q4" s="34">
+      <c r="Q4" s="23">
         <v>76.973623188405782</v>
       </c>
-      <c r="R4" s="38">
+      <c r="R4" s="27">
         <v>5.5140667441408251</v>
       </c>
     </row>
@@ -1263,23 +1316,23 @@
       <c r="J5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="12"/>
-      <c r="L5" s="37">
-        <v>2</v>
-      </c>
-      <c r="M5" s="37">
-        <v>2</v>
-      </c>
-      <c r="O5" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P5" s="33" t="s">
+      <c r="K5" s="34"/>
+      <c r="L5" s="26">
+        <v>1</v>
+      </c>
+      <c r="M5" s="26">
+        <v>1</v>
+      </c>
+      <c r="O5" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P5" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="Q5" s="34">
+      <c r="Q5" s="23">
         <v>73.133043478260859</v>
       </c>
-      <c r="R5" s="38">
+      <c r="R5" s="27">
         <v>11.796733410807491</v>
       </c>
     </row>
@@ -1314,23 +1367,23 @@
       <c r="J6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="12"/>
-      <c r="L6" s="37">
-        <v>2</v>
-      </c>
-      <c r="M6" s="37">
-        <v>2</v>
-      </c>
-      <c r="O6" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P6" s="33" t="s">
+      <c r="K6" s="34"/>
+      <c r="L6" s="26">
+        <v>1</v>
+      </c>
+      <c r="M6" s="26">
+        <v>1</v>
+      </c>
+      <c r="O6" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P6" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="Q6" s="34">
+      <c r="Q6" s="23">
         <v>72.915652173913045</v>
       </c>
-      <c r="R6" s="38">
+      <c r="R6" s="27">
         <v>4.7794000774741585</v>
       </c>
     </row>
@@ -1365,27 +1418,27 @@
       <c r="J7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="12"/>
-      <c r="L7" s="37">
-        <v>2</v>
-      </c>
-      <c r="M7" s="37">
-        <v>2</v>
-      </c>
-      <c r="O7" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P7" s="33" t="s">
+      <c r="K7" s="34"/>
+      <c r="L7" s="26">
+        <v>1</v>
+      </c>
+      <c r="M7" s="26">
+        <v>1</v>
+      </c>
+      <c r="O7" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P7" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="Q7" s="34">
+      <c r="Q7" s="23">
         <v>76.228695652173911</v>
       </c>
-      <c r="R7" s="38">
+      <c r="R7" s="27">
         <v>4.4727334108074919</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1416,27 +1469,29 @@
       <c r="J8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="13"/>
-      <c r="L8" s="37">
-        <v>2</v>
-      </c>
-      <c r="M8" s="37">
-        <v>2</v>
-      </c>
-      <c r="O8" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P8" s="33" t="s">
+      <c r="K8" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="L8" s="26">
+        <v>1</v>
+      </c>
+      <c r="M8" s="26">
+        <v>1</v>
+      </c>
+      <c r="O8" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P8" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="Q8" s="34">
+      <c r="Q8" s="23">
         <v>47.901159420289858</v>
       </c>
-      <c r="R8" s="38">
+      <c r="R8" s="27">
         <v>22.771400077474162</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -1467,29 +1522,29 @@
       <c r="J9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L9" s="37">
-        <v>2</v>
-      </c>
-      <c r="M9" s="37">
-        <v>2</v>
-      </c>
-      <c r="O9" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P9" s="33" t="s">
+      <c r="K9" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="L9" s="26">
+        <v>1</v>
+      </c>
+      <c r="M9" s="26">
+        <v>1</v>
+      </c>
+      <c r="O9" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P9" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="Q9" s="34">
+      <c r="Q9" s="23">
         <v>47.834492753623174</v>
       </c>
-      <c r="R9" s="38">
+      <c r="R9" s="27">
         <v>22.795400077474156</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
@@ -1520,27 +1575,29 @@
       <c r="J10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="13"/>
-      <c r="L10" s="37">
-        <v>2</v>
-      </c>
-      <c r="M10" s="37">
-        <v>2</v>
-      </c>
-      <c r="O10" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P10" s="33" t="s">
+      <c r="K10" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="L10" s="26">
+        <v>3</v>
+      </c>
+      <c r="M10" s="26">
+        <v>3</v>
+      </c>
+      <c r="O10" s="29">
+        <v>46134</v>
+      </c>
+      <c r="P10" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="Q10" s="34">
+      <c r="Q10" s="31">
         <v>62.486666666666665</v>
       </c>
-      <c r="R10" s="38">
+      <c r="R10" s="32">
         <v>12.448733410807492</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -1571,27 +1628,29 @@
       <c r="J11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K11" s="13"/>
-      <c r="L11" s="37">
-        <v>2</v>
-      </c>
-      <c r="M11" s="37">
-        <v>2</v>
-      </c>
-      <c r="O11" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P11" s="33" t="s">
+      <c r="K11" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="L11" s="26">
+        <v>4</v>
+      </c>
+      <c r="M11" s="26">
+        <v>4</v>
+      </c>
+      <c r="O11" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P11" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="Q11" s="34">
+      <c r="Q11" s="23">
         <v>89.509855072463765</v>
       </c>
-      <c r="R11" s="38">
+      <c r="R11" s="27">
         <v>7.3034000774741594</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -1622,23 +1681,25 @@
       <c r="J12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="13"/>
-      <c r="L12" s="37">
-        <v>2</v>
-      </c>
-      <c r="M12" s="37">
-        <v>2</v>
-      </c>
-      <c r="O12" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P12" s="33" t="s">
+      <c r="K12" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="L12" s="26">
+        <v>4</v>
+      </c>
+      <c r="M12" s="26">
+        <v>3</v>
+      </c>
+      <c r="O12" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P12" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="Q12" s="34">
+      <c r="Q12" s="23">
         <v>77.275072463768097</v>
       </c>
-      <c r="R12" s="38">
+      <c r="R12" s="27">
         <v>4.5247334108074915</v>
       </c>
     </row>
@@ -1673,23 +1734,23 @@
       <c r="J13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="12"/>
-      <c r="L13" s="37">
-        <v>2</v>
-      </c>
-      <c r="M13" s="37">
-        <v>2</v>
-      </c>
-      <c r="O13" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P13" s="33" t="s">
+      <c r="K13" s="34"/>
+      <c r="L13" s="26">
+        <v>1</v>
+      </c>
+      <c r="M13" s="26">
+        <v>1</v>
+      </c>
+      <c r="O13" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P13" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="Q13" s="34">
+      <c r="Q13" s="23">
         <v>48.159130434782604</v>
       </c>
-      <c r="R13" s="38">
+      <c r="R13" s="27">
         <v>21.938066744140819</v>
       </c>
     </row>
@@ -1724,25 +1785,25 @@
       <c r="J14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K14" s="12" t="s">
+      <c r="K14" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="L14" s="37">
-        <v>2</v>
-      </c>
-      <c r="M14" s="37">
-        <v>2</v>
-      </c>
-      <c r="O14" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P14" s="33" t="s">
+      <c r="L14" s="26">
+        <v>1</v>
+      </c>
+      <c r="M14" s="26">
+        <v>1</v>
+      </c>
+      <c r="O14" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P14" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="Q14" s="34">
+      <c r="Q14" s="23">
         <v>46.396811594202887</v>
       </c>
-      <c r="R14" s="38">
+      <c r="R14" s="27">
         <v>21.803400077474159</v>
       </c>
     </row>
@@ -1777,23 +1838,23 @@
       <c r="J15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="12"/>
-      <c r="L15" s="37">
-        <v>2</v>
-      </c>
-      <c r="M15" s="37">
-        <v>2</v>
-      </c>
-      <c r="O15" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P15" s="33" t="s">
+      <c r="K15" s="34"/>
+      <c r="L15" s="26">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <v>1</v>
+      </c>
+      <c r="O15" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P15" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="Q15" s="34">
+      <c r="Q15" s="31">
         <v>53.014202898550721</v>
       </c>
-      <c r="R15" s="38">
+      <c r="R15" s="32">
         <v>13.702066744140826</v>
       </c>
     </row>
@@ -1828,23 +1889,23 @@
       <c r="J16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="12"/>
-      <c r="L16" s="37">
-        <v>2</v>
-      </c>
-      <c r="M16" s="37">
-        <v>2</v>
-      </c>
-      <c r="O16" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P16" s="33" t="s">
+      <c r="K16" s="34"/>
+      <c r="L16" s="26">
+        <v>1</v>
+      </c>
+      <c r="M16" s="26">
+        <v>1</v>
+      </c>
+      <c r="O16" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P16" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="Q16" s="34">
+      <c r="Q16" s="23">
         <v>70.162028985507249</v>
       </c>
-      <c r="R16" s="38">
+      <c r="R16" s="27">
         <v>4.7674000774741589</v>
       </c>
     </row>
@@ -1879,23 +1940,23 @@
       <c r="J17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="12"/>
-      <c r="L17" s="37">
-        <v>2</v>
-      </c>
-      <c r="M17" s="37">
-        <v>2</v>
-      </c>
-      <c r="O17" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P17" s="33" t="s">
+      <c r="K17" s="34"/>
+      <c r="L17" s="26">
+        <v>1</v>
+      </c>
+      <c r="M17" s="26">
+        <v>1</v>
+      </c>
+      <c r="O17" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P17" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="Q17" s="34">
+      <c r="Q17" s="23">
         <v>71.799710144927531</v>
       </c>
-      <c r="R17" s="38">
+      <c r="R17" s="27">
         <v>4.6740667441408252</v>
       </c>
     </row>
@@ -1930,27 +1991,27 @@
       <c r="J18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="13"/>
-      <c r="L18" s="37">
-        <v>2</v>
-      </c>
-      <c r="M18" s="37">
-        <v>2</v>
-      </c>
-      <c r="O18" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P18" s="33" t="s">
+      <c r="K18" s="35"/>
+      <c r="L18" s="26">
+        <v>1</v>
+      </c>
+      <c r="M18" s="26">
+        <v>1</v>
+      </c>
+      <c r="O18" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P18" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="Q18" s="34">
+      <c r="Q18" s="23">
         <v>68.680869565217378</v>
       </c>
-      <c r="R18" s="38">
+      <c r="R18" s="27">
         <v>12.278066744140826</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>24</v>
       </c>
@@ -1981,27 +2042,29 @@
       <c r="J19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K19" s="13"/>
-      <c r="L19" s="37">
-        <v>2</v>
-      </c>
-      <c r="M19" s="37">
-        <v>2</v>
-      </c>
-      <c r="O19" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P19" s="33" t="s">
+      <c r="K19" s="35" t="s">
+        <v>156</v>
+      </c>
+      <c r="L19" s="26">
+        <v>4</v>
+      </c>
+      <c r="M19" s="26">
+        <v>3</v>
+      </c>
+      <c r="O19" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P19" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="Q19" s="34">
+      <c r="Q19" s="23">
         <v>81.915652173913045</v>
       </c>
-      <c r="R19" s="38">
+      <c r="R19" s="27">
         <v>4.7527334108074921</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
@@ -2032,23 +2095,25 @@
       <c r="J20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K20" s="13"/>
-      <c r="L20" s="37">
-        <v>2</v>
-      </c>
-      <c r="M20" s="37">
-        <v>2</v>
-      </c>
-      <c r="O20" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P20" s="33" t="s">
+      <c r="K20" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="L20" s="26">
+        <v>3</v>
+      </c>
+      <c r="M20" s="26">
+        <v>3</v>
+      </c>
+      <c r="O20" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P20" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="Q20" s="34">
+      <c r="Q20" s="23">
         <v>73.301159420289864</v>
       </c>
-      <c r="R20" s="38">
+      <c r="R20" s="27">
         <v>4.9940667441408255</v>
       </c>
     </row>
@@ -2083,23 +2148,23 @@
       <c r="J21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="12"/>
-      <c r="L21" s="37">
-        <v>2</v>
-      </c>
-      <c r="M21" s="37">
-        <v>2</v>
-      </c>
-      <c r="O21" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P21" s="33" t="s">
+      <c r="K21" s="34"/>
+      <c r="L21" s="26">
+        <v>1</v>
+      </c>
+      <c r="M21" s="26">
+        <v>1</v>
+      </c>
+      <c r="O21" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P21" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="Q21" s="34">
+      <c r="Q21" s="23">
         <v>51.121449275362323</v>
       </c>
-      <c r="R21" s="38">
+      <c r="R21" s="27">
         <v>20.847400077474155</v>
       </c>
     </row>
@@ -2134,23 +2199,23 @@
       <c r="J22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K22" s="12"/>
-      <c r="L22" s="37">
-        <v>2</v>
-      </c>
-      <c r="M22" s="37">
-        <v>2</v>
-      </c>
-      <c r="O22" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P22" s="33" t="s">
+      <c r="K22" s="34"/>
+      <c r="L22" s="26">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26">
+        <v>1</v>
+      </c>
+      <c r="O22" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P22" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="Q22" s="34">
+      <c r="Q22" s="23">
         <v>60.892463768115938</v>
       </c>
-      <c r="R22" s="38">
+      <c r="R22" s="27">
         <v>13.186066744140827</v>
       </c>
     </row>
@@ -2185,23 +2250,23 @@
       <c r="J23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K23" s="12"/>
-      <c r="L23" s="37">
-        <v>2</v>
-      </c>
-      <c r="M23" s="37">
-        <v>2</v>
-      </c>
-      <c r="O23" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P23" s="33" t="s">
+      <c r="K23" s="34"/>
+      <c r="L23" s="26">
+        <v>1</v>
+      </c>
+      <c r="M23" s="26">
+        <v>1</v>
+      </c>
+      <c r="O23" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P23" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="Q23" s="34">
+      <c r="Q23" s="23">
         <v>70.901159420289844</v>
       </c>
-      <c r="R23" s="38">
+      <c r="R23" s="27">
         <v>3.6894000774741582</v>
       </c>
     </row>
@@ -2236,25 +2301,25 @@
       <c r="J24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="K24" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="L24" s="37">
-        <v>2</v>
-      </c>
-      <c r="M24" s="37">
-        <v>2</v>
-      </c>
-      <c r="O24" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P24" s="33" t="s">
+      <c r="L24" s="26">
+        <v>1</v>
+      </c>
+      <c r="M24" s="26">
+        <v>1</v>
+      </c>
+      <c r="O24" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P24" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="Q24" s="34">
+      <c r="Q24" s="23">
         <v>70.993913043478244</v>
       </c>
-      <c r="R24" s="38">
+      <c r="R24" s="27">
         <v>4.7327334108074925</v>
       </c>
     </row>
@@ -2289,23 +2354,23 @@
       <c r="J25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K25" s="12"/>
-      <c r="L25" s="37">
-        <v>2</v>
-      </c>
-      <c r="M25" s="37">
-        <v>2</v>
-      </c>
-      <c r="O25" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P25" s="33" t="s">
+      <c r="K25" s="34"/>
+      <c r="L25" s="26">
+        <v>1</v>
+      </c>
+      <c r="M25" s="26">
+        <v>1</v>
+      </c>
+      <c r="O25" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P25" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="Q25" s="34">
+      <c r="Q25" s="23">
         <v>70.327246376811587</v>
       </c>
-      <c r="R25" s="38">
+      <c r="R25" s="27">
         <v>4.4220667441408255</v>
       </c>
     </row>
@@ -2340,23 +2405,23 @@
       <c r="J26" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K26" s="13"/>
-      <c r="L26" s="37">
-        <v>2</v>
-      </c>
-      <c r="M26" s="37">
-        <v>2</v>
-      </c>
-      <c r="O26" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P26" s="32" t="s">
+      <c r="K26" s="35"/>
+      <c r="L26" s="26">
+        <v>1</v>
+      </c>
+      <c r="M26" s="26">
+        <v>1</v>
+      </c>
+      <c r="O26" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P26" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="Q26" s="34">
+      <c r="Q26" s="23">
         <v>58.101159420289846</v>
       </c>
-      <c r="R26" s="38">
+      <c r="R26" s="27">
         <v>16.050066744140821</v>
       </c>
     </row>
@@ -2391,23 +2456,23 @@
       <c r="J27" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K27" s="13"/>
-      <c r="L27" s="37">
-        <v>2</v>
-      </c>
-      <c r="M27" s="37">
-        <v>2</v>
-      </c>
-      <c r="O27" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P27" s="32" t="s">
+      <c r="K27" s="35"/>
+      <c r="L27" s="26">
+        <v>1</v>
+      </c>
+      <c r="M27" s="26">
+        <v>1</v>
+      </c>
+      <c r="O27" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P27" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="Q27" s="34">
+      <c r="Q27" s="23">
         <v>74.817101449275356</v>
       </c>
-      <c r="R27" s="38">
+      <c r="R27" s="27">
         <v>5.3180667441408245</v>
       </c>
     </row>
@@ -2442,23 +2507,23 @@
       <c r="J28" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K28" s="13"/>
-      <c r="L28" s="37">
-        <v>2</v>
-      </c>
-      <c r="M28" s="37">
-        <v>2</v>
-      </c>
-      <c r="O28" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P28" s="32" t="s">
+      <c r="K28" s="35"/>
+      <c r="L28" s="26">
+        <v>1</v>
+      </c>
+      <c r="M28" s="26">
+        <v>1</v>
+      </c>
+      <c r="O28" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P28" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="Q28" s="34">
+      <c r="Q28" s="23">
         <v>76.843188405797093</v>
       </c>
-      <c r="R28" s="38">
+      <c r="R28" s="27">
         <v>4.1527334108074916</v>
       </c>
     </row>
@@ -2493,23 +2558,23 @@
       <c r="J29" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K29" s="12"/>
-      <c r="L29" s="37">
-        <v>2</v>
-      </c>
-      <c r="M29" s="37">
-        <v>2</v>
-      </c>
-      <c r="O29" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P29" s="32" t="s">
+      <c r="K29" s="34"/>
+      <c r="L29" s="26">
+        <v>1</v>
+      </c>
+      <c r="M29" s="26">
+        <v>1</v>
+      </c>
+      <c r="O29" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P29" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="Q29" s="34">
+      <c r="Q29" s="23">
         <v>53.8431884057971</v>
       </c>
-      <c r="R29" s="38">
+      <c r="R29" s="27">
         <v>19.85406674414083</v>
       </c>
     </row>
@@ -2544,23 +2609,23 @@
       <c r="J30" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K30" s="12"/>
-      <c r="L30" s="37">
-        <v>2</v>
-      </c>
-      <c r="M30" s="37">
-        <v>2</v>
-      </c>
-      <c r="O30" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P30" s="32" t="s">
+      <c r="K30" s="34"/>
+      <c r="L30" s="26">
+        <v>1</v>
+      </c>
+      <c r="M30" s="26">
+        <v>1</v>
+      </c>
+      <c r="O30" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P30" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="Q30" s="34">
+      <c r="Q30" s="23">
         <v>56.933043478260871</v>
       </c>
-      <c r="R30" s="38">
+      <c r="R30" s="27">
         <v>14.314066744140828</v>
       </c>
     </row>
@@ -2595,23 +2660,23 @@
       <c r="J31" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K31" s="12"/>
-      <c r="L31" s="37">
-        <v>2</v>
-      </c>
-      <c r="M31" s="37">
-        <v>2</v>
-      </c>
-      <c r="O31" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P31" s="32" t="s">
+      <c r="K31" s="34"/>
+      <c r="L31" s="26">
+        <v>1</v>
+      </c>
+      <c r="M31" s="26">
+        <v>1</v>
+      </c>
+      <c r="O31" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P31" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="Q31" s="34">
+      <c r="Q31" s="23">
         <v>68.02</v>
       </c>
-      <c r="R31" s="38">
+      <c r="R31" s="27">
         <v>6.998066744140826</v>
       </c>
     </row>
@@ -2646,23 +2711,23 @@
       <c r="J32" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K32" s="12"/>
-      <c r="L32" s="37">
-        <v>2</v>
-      </c>
-      <c r="M32" s="37">
-        <v>2</v>
-      </c>
-      <c r="O32" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P32" s="32" t="s">
+      <c r="K32" s="34"/>
+      <c r="L32" s="26">
+        <v>1</v>
+      </c>
+      <c r="M32" s="26">
+        <v>1</v>
+      </c>
+      <c r="O32" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P32" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="Q32" s="34">
+      <c r="Q32" s="23">
         <v>72.535942028985502</v>
       </c>
-      <c r="R32" s="38">
+      <c r="R32" s="27">
         <v>4.2980667441408249</v>
       </c>
     </row>
@@ -2697,23 +2762,23 @@
       <c r="J33" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K33" s="13"/>
-      <c r="L33" s="37">
-        <v>2</v>
-      </c>
-      <c r="M33" s="37">
-        <v>2</v>
-      </c>
-      <c r="O33" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P33" s="32" t="s">
+      <c r="K33" s="35"/>
+      <c r="L33" s="26">
+        <v>1</v>
+      </c>
+      <c r="M33" s="26">
+        <v>1</v>
+      </c>
+      <c r="O33" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P33" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="Q33" s="34">
+      <c r="Q33" s="23">
         <v>79.683768115942016</v>
       </c>
-      <c r="R33" s="38">
+      <c r="R33" s="27">
         <v>4.7100667441408257</v>
       </c>
     </row>
@@ -2748,23 +2813,23 @@
       <c r="J34" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K34" s="13"/>
-      <c r="L34" s="37">
-        <v>2</v>
-      </c>
-      <c r="M34" s="37">
-        <v>2</v>
-      </c>
-      <c r="O34" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P34" s="32" t="s">
+      <c r="K34" s="35"/>
+      <c r="L34" s="26">
+        <v>1</v>
+      </c>
+      <c r="M34" s="26">
+        <v>1</v>
+      </c>
+      <c r="O34" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P34" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="Q34" s="34">
+      <c r="Q34" s="23">
         <v>85.075072463768123</v>
       </c>
-      <c r="R34" s="38">
+      <c r="R34" s="27">
         <v>5.1754000774741593</v>
       </c>
     </row>
@@ -2799,27 +2864,27 @@
       <c r="J35" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K35" s="12"/>
-      <c r="L35" s="37">
-        <v>2</v>
-      </c>
-      <c r="M35" s="37">
-        <v>2</v>
-      </c>
-      <c r="O35" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P35" s="32" t="s">
+      <c r="K35" s="34"/>
+      <c r="L35" s="26">
+        <v>1</v>
+      </c>
+      <c r="M35" s="26">
+        <v>1</v>
+      </c>
+      <c r="O35" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P35" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="Q35" s="34">
+      <c r="Q35" s="23">
         <v>86.727246376811593</v>
       </c>
-      <c r="R35" s="38">
+      <c r="R35" s="27">
         <v>4.9647334108074919</v>
       </c>
     </row>
-    <row r="36" spans="1:18" s="30" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" s="19" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>24</v>
       </c>
@@ -2850,23 +2915,23 @@
       <c r="J36" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K36" s="14"/>
-      <c r="L36" s="37">
-        <v>2</v>
-      </c>
-      <c r="M36" s="37">
-        <v>2</v>
-      </c>
-      <c r="O36" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P36" s="31" t="s">
+      <c r="K36" s="36"/>
+      <c r="L36" s="26">
+        <v>1</v>
+      </c>
+      <c r="M36" s="26">
+        <v>1</v>
+      </c>
+      <c r="O36" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P36" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="Q36" s="35">
+      <c r="Q36" s="24">
         <v>90.756231884057968</v>
       </c>
-      <c r="R36" s="38">
+      <c r="R36" s="27">
         <v>5.5660667441408247</v>
       </c>
     </row>
@@ -2901,23 +2966,23 @@
       <c r="J37" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="K37" s="15"/>
-      <c r="L37" s="37">
-        <v>2</v>
-      </c>
-      <c r="M37" s="37">
-        <v>2</v>
-      </c>
-      <c r="O37" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P37" s="32" t="s">
+      <c r="K37" s="37"/>
+      <c r="L37" s="26">
+        <v>1</v>
+      </c>
+      <c r="M37" s="26">
+        <v>1</v>
+      </c>
+      <c r="O37" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P37" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="Q37" s="34">
+      <c r="Q37" s="23">
         <v>94.263287548045</v>
       </c>
-      <c r="R37" s="38">
+      <c r="R37" s="27">
         <v>6.6093979441997073</v>
       </c>
     </row>
@@ -2952,27 +3017,27 @@
       <c r="J38" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="37">
-        <v>2</v>
-      </c>
-      <c r="M38" s="37">
-        <v>2</v>
-      </c>
-      <c r="O38" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P38" s="32" t="s">
+      <c r="K38" s="11"/>
+      <c r="L38" s="26">
+        <v>1</v>
+      </c>
+      <c r="M38" s="26">
+        <v>1</v>
+      </c>
+      <c r="O38" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P38" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="Q38" s="34">
+      <c r="Q38" s="23">
         <v>89.695819787935335</v>
       </c>
-      <c r="R38" s="38">
+      <c r="R38" s="27">
         <v>5.5124816446402347</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="29.25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>26</v>
       </c>
@@ -3003,29 +3068,29 @@
       <c r="J39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K39" s="17" t="s">
+      <c r="K39" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="L39" s="37">
-        <v>2</v>
-      </c>
-      <c r="M39" s="37">
-        <v>2</v>
-      </c>
-      <c r="O39" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P39" s="32" t="s">
+      <c r="L39" s="26">
+        <v>1</v>
+      </c>
+      <c r="M39" s="26">
+        <v>1</v>
+      </c>
+      <c r="O39" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P39" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="Q39" s="34">
+      <c r="Q39" s="23">
         <v>77.349646198338263</v>
       </c>
-      <c r="R39" s="38">
+      <c r="R39" s="27">
         <v>6.0719530102790005</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="43.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>26</v>
       </c>
@@ -3056,25 +3121,25 @@
       <c r="J40" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K40" s="17" t="s">
+      <c r="K40" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="L40" s="37">
-        <v>2</v>
-      </c>
-      <c r="M40" s="37">
-        <v>2</v>
-      </c>
-      <c r="O40" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P40" s="32" t="s">
+      <c r="L40" s="26">
+        <v>1</v>
+      </c>
+      <c r="M40" s="26">
+        <v>1</v>
+      </c>
+      <c r="O40" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P40" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="Q40" s="34">
+      <c r="Q40" s="23">
         <v>76.733178157096475</v>
       </c>
-      <c r="R40" s="38">
+      <c r="R40" s="27">
         <v>6.1027900146842873</v>
       </c>
     </row>
@@ -3109,23 +3174,23 @@
       <c r="J41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K41" s="17"/>
-      <c r="L41" s="37">
-        <v>2</v>
-      </c>
-      <c r="M41" s="37">
-        <v>2</v>
-      </c>
-      <c r="O41" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P41" s="32" t="s">
+      <c r="K41" s="38"/>
+      <c r="L41" s="26">
+        <v>1</v>
+      </c>
+      <c r="M41" s="26">
+        <v>1</v>
+      </c>
+      <c r="O41" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P41" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="Q41" s="34">
+      <c r="Q41" s="23">
         <v>82.88665005967367</v>
       </c>
-      <c r="R41" s="38">
+      <c r="R41" s="27">
         <v>5.0748898678414101</v>
       </c>
     </row>
@@ -3160,25 +3225,25 @@
       <c r="J42" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K42" s="16" t="s">
+      <c r="K42" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L42" s="37">
-        <v>2</v>
-      </c>
-      <c r="M42" s="37">
-        <v>2</v>
-      </c>
-      <c r="O42" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P42" s="32" t="s">
+      <c r="L42" s="26">
+        <v>1</v>
+      </c>
+      <c r="M42" s="26">
+        <v>1</v>
+      </c>
+      <c r="O42" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P42" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="Q42" s="34">
+      <c r="Q42" s="23">
         <v>78.588186535742238</v>
       </c>
-      <c r="R42" s="38">
+      <c r="R42" s="27">
         <v>5.4170337738619674</v>
       </c>
     </row>
@@ -3213,23 +3278,23 @@
       <c r="J43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="37">
-        <v>2</v>
-      </c>
-      <c r="M43" s="37">
-        <v>2</v>
-      </c>
-      <c r="O43" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P43" s="32" t="s">
+      <c r="K43" s="11"/>
+      <c r="L43" s="26">
+        <v>1</v>
+      </c>
+      <c r="M43" s="26">
+        <v>1</v>
+      </c>
+      <c r="O43" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P43" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="Q43" s="34">
+      <c r="Q43" s="23">
         <v>81.230592730701417</v>
       </c>
-      <c r="R43" s="38">
+      <c r="R43" s="27">
         <v>5.0998531571218795</v>
       </c>
     </row>
@@ -3264,23 +3329,23 @@
       <c r="J44" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K44" s="17"/>
-      <c r="L44" s="37">
-        <v>2</v>
-      </c>
-      <c r="M44" s="37">
-        <v>2</v>
-      </c>
-      <c r="O44" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P44" s="32" t="s">
+      <c r="K44" s="38"/>
+      <c r="L44" s="26">
+        <v>1</v>
+      </c>
+      <c r="M44" s="26">
+        <v>1</v>
+      </c>
+      <c r="O44" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P44" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="Q44" s="34">
+      <c r="Q44" s="23">
         <v>46.50943137148731</v>
       </c>
-      <c r="R44" s="38">
+      <c r="R44" s="27">
         <v>22.390602055800287</v>
       </c>
     </row>
@@ -3315,23 +3380,23 @@
       <c r="J45" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K45" s="17"/>
-      <c r="L45" s="37">
-        <v>2</v>
-      </c>
-      <c r="M45" s="37">
-        <v>2</v>
-      </c>
-      <c r="O45" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P45" s="32" t="s">
+      <c r="K45" s="38"/>
+      <c r="L45" s="26">
+        <v>1</v>
+      </c>
+      <c r="M45" s="26">
+        <v>1</v>
+      </c>
+      <c r="O45" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P45" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="Q45" s="34">
+      <c r="Q45" s="23">
         <v>51.73820121220183</v>
       </c>
-      <c r="R45" s="38">
+      <c r="R45" s="27">
         <v>15.01468428781204</v>
       </c>
     </row>
@@ -3366,23 +3431,23 @@
       <c r="J46" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K46" s="17"/>
-      <c r="L46" s="37">
-        <v>2</v>
-      </c>
-      <c r="M46" s="37">
-        <v>2</v>
-      </c>
-      <c r="O46" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P46" s="32" t="s">
+      <c r="K46" s="38"/>
+      <c r="L46" s="26">
+        <v>1</v>
+      </c>
+      <c r="M46" s="26">
+        <v>1</v>
+      </c>
+      <c r="O46" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P46" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="Q46" s="34">
+      <c r="Q46" s="23">
         <v>69.895987154232913</v>
       </c>
-      <c r="R46" s="38">
+      <c r="R46" s="27">
         <v>5.035242290748899</v>
       </c>
     </row>
@@ -3417,23 +3482,23 @@
       <c r="J47" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K47" s="17"/>
-      <c r="L47" s="37">
-        <v>2</v>
-      </c>
-      <c r="M47" s="37">
-        <v>2</v>
-      </c>
-      <c r="O47" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P47" s="32" t="s">
+      <c r="K47" s="38"/>
+      <c r="L47" s="26">
+        <v>1</v>
+      </c>
+      <c r="M47" s="26">
+        <v>1</v>
+      </c>
+      <c r="O47" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P47" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="Q47" s="34">
+      <c r="Q47" s="23">
         <v>75.592712280799162</v>
       </c>
-      <c r="R47" s="38">
+      <c r="R47" s="27">
         <v>4.4455212922173279</v>
       </c>
     </row>
@@ -3468,23 +3533,23 @@
       <c r="J48" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="37">
-        <v>2</v>
-      </c>
-      <c r="M48" s="37">
-        <v>2</v>
-      </c>
-      <c r="O48" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P48" s="32" t="s">
+      <c r="K48" s="11"/>
+      <c r="L48" s="26">
+        <v>1</v>
+      </c>
+      <c r="M48" s="26">
+        <v>1</v>
+      </c>
+      <c r="O48" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P48" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="Q48" s="34">
+      <c r="Q48" s="23">
         <v>49.706658803564096</v>
       </c>
-      <c r="R48" s="38">
+      <c r="R48" s="27">
         <v>21.883994126284872</v>
       </c>
     </row>
@@ -3519,25 +3584,25 @@
       <c r="J49" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K49" s="16" t="s">
+      <c r="K49" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="L49" s="37">
-        <v>2</v>
-      </c>
-      <c r="M49" s="37">
-        <v>2</v>
-      </c>
-      <c r="O49" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P49" s="32" t="s">
+      <c r="L49" s="26">
+        <v>1</v>
+      </c>
+      <c r="M49" s="26">
+        <v>1</v>
+      </c>
+      <c r="O49" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P49" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="Q49" s="34">
+      <c r="Q49" s="23">
         <v>49.605782214997248</v>
       </c>
-      <c r="R49" s="39">
+      <c r="R49" s="28">
         <v>23.400881057268723</v>
       </c>
     </row>
@@ -3572,23 +3637,23 @@
       <c r="J50" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="37">
-        <v>2</v>
-      </c>
-      <c r="M50" s="37">
-        <v>2</v>
-      </c>
-      <c r="O50" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P50" s="32" t="s">
+      <c r="K50" s="11"/>
+      <c r="L50" s="26">
+        <v>1</v>
+      </c>
+      <c r="M50" s="26">
+        <v>1</v>
+      </c>
+      <c r="O50" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P50" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="Q50" s="34">
+      <c r="Q50" s="23">
         <v>52.122092674247853</v>
       </c>
-      <c r="R50" s="38">
+      <c r="R50" s="27">
         <v>14.906020558002936</v>
       </c>
     </row>
@@ -3623,27 +3688,27 @@
       <c r="J51" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="37">
-        <v>2</v>
-      </c>
-      <c r="M51" s="37">
-        <v>2</v>
-      </c>
-      <c r="O51" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P51" s="32" t="s">
+      <c r="K51" s="11"/>
+      <c r="L51" s="26">
+        <v>1</v>
+      </c>
+      <c r="M51" s="26">
+        <v>1</v>
+      </c>
+      <c r="O51" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P51" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Q51" s="34">
+      <c r="Q51" s="23">
         <v>72.650478447599667</v>
       </c>
-      <c r="R51" s="38">
+      <c r="R51" s="27">
         <v>6.3715124816446407</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>26</v>
       </c>
@@ -3674,23 +3739,25 @@
       <c r="J52" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="37">
-        <v>2</v>
-      </c>
-      <c r="M52" s="37">
-        <v>2</v>
-      </c>
-      <c r="O52" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P52" s="32" t="s">
+      <c r="K52" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="L52" s="26">
+        <v>3</v>
+      </c>
+      <c r="M52" s="26">
+        <v>1</v>
+      </c>
+      <c r="O52" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P52" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="Q52" s="34">
-        <v>82.712918157141885</v>
-      </c>
-      <c r="R52" s="38">
+      <c r="Q52" s="23">
+        <v>82.7129181571419</v>
+      </c>
+      <c r="R52" s="27">
         <v>4.7283406754772388</v>
       </c>
     </row>
@@ -3725,23 +3792,23 @@
       <c r="J53" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K53" s="17"/>
-      <c r="L53" s="37">
-        <v>2</v>
-      </c>
-      <c r="M53" s="37">
-        <v>2</v>
-      </c>
-      <c r="O53" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P53" s="32" t="s">
+      <c r="K53" s="38"/>
+      <c r="L53" s="26">
+        <v>1</v>
+      </c>
+      <c r="M53" s="26">
+        <v>1</v>
+      </c>
+      <c r="O53" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P53" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="Q53" s="34">
+      <c r="Q53" s="23">
         <v>62.094864305064007</v>
       </c>
-      <c r="R53" s="38">
+      <c r="R53" s="27">
         <v>11.669603524229075</v>
       </c>
     </row>
@@ -3776,23 +3843,23 @@
       <c r="J54" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K54" s="17"/>
-      <c r="L54" s="37">
-        <v>2</v>
-      </c>
-      <c r="M54" s="37">
-        <v>2</v>
-      </c>
-      <c r="O54" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P54" s="32" t="s">
+      <c r="K54" s="38"/>
+      <c r="L54" s="26">
+        <v>1</v>
+      </c>
+      <c r="M54" s="26">
+        <v>1</v>
+      </c>
+      <c r="O54" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P54" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="Q54" s="34">
+      <c r="Q54" s="23">
         <v>70.072521184224883</v>
       </c>
-      <c r="R54" s="38">
+      <c r="R54" s="27">
         <v>7.7459618208516874</v>
       </c>
     </row>
@@ -3827,23 +3894,23 @@
       <c r="J55" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K55" s="17"/>
-      <c r="L55" s="37">
-        <v>2</v>
-      </c>
-      <c r="M55" s="37">
-        <v>2</v>
-      </c>
-      <c r="O55" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P55" s="32" t="s">
+      <c r="K55" s="38"/>
+      <c r="L55" s="26">
+        <v>1</v>
+      </c>
+      <c r="M55" s="26">
+        <v>1</v>
+      </c>
+      <c r="O55" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P55" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="Q55" s="34">
+      <c r="Q55" s="23">
         <v>80.807471484212712</v>
       </c>
-      <c r="R55" s="38">
+      <c r="R55" s="27">
         <v>5.2804698972099855</v>
       </c>
     </row>
@@ -3878,27 +3945,27 @@
       <c r="J56" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="37">
-        <v>2</v>
-      </c>
-      <c r="M56" s="37">
-        <v>2</v>
-      </c>
-      <c r="O56" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P56" s="32" t="s">
+      <c r="K56" s="11"/>
+      <c r="L56" s="26">
+        <v>1</v>
+      </c>
+      <c r="M56" s="26">
+        <v>1</v>
+      </c>
+      <c r="O56" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P56" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="Q56" s="34">
+      <c r="Q56" s="23">
         <v>53.890235101627738</v>
       </c>
-      <c r="R56" s="38">
+      <c r="R56" s="27">
         <v>15.580029368575623</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="72" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>26</v>
       </c>
@@ -3929,25 +3996,25 @@
       <c r="J57" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K57" s="16" t="s">
+      <c r="K57" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="L57" s="37">
-        <v>2</v>
-      </c>
-      <c r="M57" s="37">
-        <v>2</v>
-      </c>
-      <c r="O57" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P57" s="32" t="s">
+      <c r="L57" s="26">
+        <v>1</v>
+      </c>
+      <c r="M57" s="26">
+        <v>1</v>
+      </c>
+      <c r="O57" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P57" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="Q57" s="34">
+      <c r="Q57" s="23">
         <v>58.970492186952171</v>
       </c>
-      <c r="R57" s="38">
+      <c r="R57" s="27">
         <v>12.745961820851686</v>
       </c>
     </row>
@@ -3982,23 +4049,23 @@
       <c r="J58" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="37">
-        <v>2</v>
-      </c>
-      <c r="M58" s="37">
-        <v>2</v>
-      </c>
-      <c r="O58" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P58" s="32" t="s">
+      <c r="K58" s="11"/>
+      <c r="L58" s="26">
+        <v>1</v>
+      </c>
+      <c r="M58" s="26">
+        <v>1</v>
+      </c>
+      <c r="O58" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P58" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="Q58" s="34">
+      <c r="Q58" s="23">
         <v>70.246253086756667</v>
       </c>
-      <c r="R58" s="38">
+      <c r="R58" s="27">
         <v>5.9618208516886924</v>
       </c>
     </row>
@@ -4033,27 +4100,27 @@
       <c r="J59" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="37">
-        <v>2</v>
-      </c>
-      <c r="M59" s="37">
-        <v>2</v>
-      </c>
-      <c r="O59" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P59" s="32" t="s">
+      <c r="K59" s="11"/>
+      <c r="L59" s="26">
+        <v>1</v>
+      </c>
+      <c r="M59" s="26">
+        <v>1</v>
+      </c>
+      <c r="O59" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P59" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="Q59" s="34">
+      <c r="Q59" s="23">
         <v>78.958067360487306</v>
       </c>
-      <c r="R59" s="38">
+      <c r="R59" s="27">
         <v>4.8091042584434645</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="29.25" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>26</v>
       </c>
@@ -4084,25 +4151,25 @@
       <c r="J60" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K60" s="16" t="s">
+      <c r="K60" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="L60" s="37">
-        <v>2</v>
-      </c>
-      <c r="M60" s="37">
-        <v>2</v>
-      </c>
-      <c r="O60" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P60" s="32" t="s">
+      <c r="L60" s="26">
+        <v>1</v>
+      </c>
+      <c r="M60" s="26">
+        <v>1</v>
+      </c>
+      <c r="O60" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P60" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="Q60" s="34">
+      <c r="Q60" s="23">
         <v>80.300286413918315</v>
       </c>
-      <c r="R60" s="38">
+      <c r="R60" s="27">
         <v>4.9118942731277535</v>
       </c>
     </row>
@@ -4137,23 +4204,23 @@
       <c r="J61" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K61" s="17"/>
-      <c r="L61" s="37">
-        <v>2</v>
-      </c>
-      <c r="M61" s="37">
-        <v>2</v>
-      </c>
-      <c r="O61" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P61" s="32" t="s">
+      <c r="K61" s="38"/>
+      <c r="L61" s="26">
+        <v>1</v>
+      </c>
+      <c r="M61" s="26">
+        <v>1</v>
+      </c>
+      <c r="O61" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P61" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="Q61" s="34">
+      <c r="Q61" s="23">
         <v>47.927307866343455</v>
       </c>
-      <c r="R61" s="38">
+      <c r="R61" s="27">
         <v>19.014684287812038</v>
       </c>
     </row>
@@ -4188,23 +4255,23 @@
       <c r="J62" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K62" s="17"/>
-      <c r="L62" s="37">
-        <v>2</v>
-      </c>
-      <c r="M62" s="37">
-        <v>2</v>
-      </c>
-      <c r="O62" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P62" s="32" t="s">
+      <c r="K62" s="38"/>
+      <c r="L62" s="26">
+        <v>1</v>
+      </c>
+      <c r="M62" s="26">
+        <v>1</v>
+      </c>
+      <c r="O62" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P62" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="Q62" s="34">
+      <c r="Q62" s="23">
         <v>58.183094370638784</v>
       </c>
-      <c r="R62" s="38">
+      <c r="R62" s="27">
         <v>12.472834067547723</v>
       </c>
     </row>
@@ -4239,23 +4306,23 @@
       <c r="J63" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K63" s="17"/>
-      <c r="L63" s="37">
-        <v>2</v>
-      </c>
-      <c r="M63" s="37">
-        <v>2</v>
-      </c>
-      <c r="O63" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P63" s="32" t="s">
+      <c r="K63" s="38"/>
+      <c r="L63" s="26">
+        <v>1</v>
+      </c>
+      <c r="M63" s="26">
+        <v>1</v>
+      </c>
+      <c r="O63" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P63" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="Q63" s="34">
+      <c r="Q63" s="23">
         <v>66.555851221686453</v>
       </c>
-      <c r="R63" s="38">
+      <c r="R63" s="27">
         <v>9.1189427312775315</v>
       </c>
     </row>
@@ -4290,23 +4357,23 @@
       <c r="J64" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K64" s="17"/>
-      <c r="L64" s="37">
-        <v>2</v>
-      </c>
-      <c r="M64" s="37">
-        <v>2</v>
-      </c>
-      <c r="O64" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P64" s="32" t="s">
+      <c r="K64" s="38"/>
+      <c r="L64" s="26">
+        <v>1</v>
+      </c>
+      <c r="M64" s="26">
+        <v>1</v>
+      </c>
+      <c r="O64" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P64" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="Q64" s="34">
+      <c r="Q64" s="23">
         <v>80.538467248034465</v>
       </c>
-      <c r="R64" s="38">
+      <c r="R64" s="27">
         <v>4.8091042584434645</v>
       </c>
     </row>
@@ -4341,29 +4408,29 @@
       <c r="J65" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K65" s="17" t="s">
+      <c r="K65" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="L65" s="37">
-        <v>2</v>
-      </c>
-      <c r="M65" s="37">
-        <v>2</v>
-      </c>
-      <c r="O65" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P65" s="32" t="s">
+      <c r="L65" s="26">
+        <v>1</v>
+      </c>
+      <c r="M65" s="26">
+        <v>1</v>
+      </c>
+      <c r="O65" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P65" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="Q65" s="34">
+      <c r="Q65" s="23">
         <v>79.672609862835756</v>
       </c>
-      <c r="R65" s="38">
+      <c r="R65" s="27">
         <v>4.8604992657856094</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="43.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>26</v>
       </c>
@@ -4394,25 +4461,25 @@
       <c r="J66" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K66" s="18" t="s">
+      <c r="K66" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="L66" s="37">
-        <v>2</v>
-      </c>
-      <c r="M66" s="37">
-        <v>2</v>
-      </c>
-      <c r="O66" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P66" s="32" t="s">
+      <c r="L66" s="26">
+        <v>1</v>
+      </c>
+      <c r="M66" s="26">
+        <v>1</v>
+      </c>
+      <c r="O66" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P66" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="Q66" s="34">
+      <c r="Q66" s="23">
         <v>56.807249787685507</v>
       </c>
-      <c r="R66" s="38">
+      <c r="R66" s="27">
         <v>13.674008810572689</v>
       </c>
     </row>
@@ -4447,23 +4514,23 @@
       <c r="J67" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K67" s="16"/>
-      <c r="L67" s="37">
-        <v>2</v>
-      </c>
-      <c r="M67" s="37">
-        <v>2</v>
-      </c>
-      <c r="O67" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P67" s="32" t="s">
+      <c r="K67" s="11"/>
+      <c r="L67" s="26">
+        <v>1</v>
+      </c>
+      <c r="M67" s="26">
+        <v>1</v>
+      </c>
+      <c r="O67" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P67" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="Q67" s="34">
+      <c r="Q67" s="23">
         <v>69.498085054885934</v>
       </c>
-      <c r="R67" s="38">
+      <c r="R67" s="27">
         <v>6.7767988252569751</v>
       </c>
     </row>
@@ -4498,23 +4565,23 @@
       <c r="J68" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K68" s="16"/>
-      <c r="L68" s="37">
-        <v>2</v>
-      </c>
-      <c r="M68" s="37">
-        <v>2</v>
-      </c>
-      <c r="O68" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P68" s="32" t="s">
+      <c r="K68" s="11"/>
+      <c r="L68" s="26">
+        <v>1</v>
+      </c>
+      <c r="M68" s="26">
+        <v>1</v>
+      </c>
+      <c r="O68" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P68" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="Q68" s="34">
+      <c r="Q68" s="23">
         <v>80.19100344297091</v>
       </c>
-      <c r="R68" s="38">
+      <c r="R68" s="27">
         <v>4.3939794419970628</v>
       </c>
     </row>
@@ -4549,23 +4616,23 @@
       <c r="J69" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K69" s="17"/>
-      <c r="L69" s="37">
-        <v>2</v>
-      </c>
-      <c r="M69" s="37">
-        <v>2</v>
-      </c>
-      <c r="O69" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P69" s="32" t="s">
+      <c r="K69" s="38"/>
+      <c r="L69" s="26">
+        <v>1</v>
+      </c>
+      <c r="M69" s="26">
+        <v>1</v>
+      </c>
+      <c r="O69" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P69" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="Q69" s="34">
+      <c r="Q69" s="23">
         <v>80.342318325821182</v>
       </c>
-      <c r="R69" s="38">
+      <c r="R69" s="27">
         <v>5.819383259911894</v>
       </c>
     </row>
@@ -4600,27 +4667,27 @@
       <c r="J70" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K70" s="17"/>
-      <c r="L70" s="37">
-        <v>2</v>
-      </c>
-      <c r="M70" s="37">
-        <v>2</v>
-      </c>
-      <c r="O70" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P70" s="32" t="s">
+      <c r="K70" s="38"/>
+      <c r="L70" s="26">
+        <v>1</v>
+      </c>
+      <c r="M70" s="26">
+        <v>1</v>
+      </c>
+      <c r="O70" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P70" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="Q70" s="34">
+      <c r="Q70" s="23">
         <v>82.032001184315732</v>
       </c>
-      <c r="R70" s="38">
+      <c r="R70" s="27">
         <v>4.3339207048458146</v>
       </c>
     </row>
-    <row r="71" spans="1:18" s="30" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" s="19" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="8" t="s">
         <v>26</v>
       </c>
@@ -4651,23 +4718,23 @@
       <c r="J71" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="K71" s="19"/>
-      <c r="L71" s="37">
-        <v>2</v>
-      </c>
-      <c r="M71" s="37">
-        <v>2</v>
-      </c>
-      <c r="O71" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P71" s="31" t="s">
+      <c r="K71" s="39"/>
+      <c r="L71" s="26">
+        <v>1</v>
+      </c>
+      <c r="M71" s="26">
+        <v>1</v>
+      </c>
+      <c r="O71" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P71" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="Q71" s="35">
+      <c r="Q71" s="24">
         <v>95.159968335305805</v>
       </c>
-      <c r="R71" s="38">
+      <c r="R71" s="27">
         <v>7.7165932452276067</v>
       </c>
     </row>
@@ -4702,23 +4769,23 @@
       <c r="J72" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="K72" s="15"/>
-      <c r="L72" s="37">
-        <v>2</v>
-      </c>
-      <c r="M72" s="37">
-        <v>2</v>
-      </c>
-      <c r="O72" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P72" s="32" t="s">
+      <c r="K72" s="37"/>
+      <c r="L72" s="26">
+        <v>1</v>
+      </c>
+      <c r="M72" s="26">
+        <v>1</v>
+      </c>
+      <c r="O72" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P72" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="Q72" s="34">
+      <c r="Q72" s="23">
         <v>96.129785029785026</v>
       </c>
-      <c r="R72" s="38">
+      <c r="R72" s="27">
         <v>9.0578386605783852</v>
       </c>
     </row>
@@ -4753,23 +4820,23 @@
       <c r="J73" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K73" s="16"/>
-      <c r="L73" s="37">
-        <v>2</v>
-      </c>
-      <c r="M73" s="37">
-        <v>2</v>
-      </c>
-      <c r="O73" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P73" s="32" t="s">
+      <c r="K73" s="11"/>
+      <c r="L73" s="26">
+        <v>1</v>
+      </c>
+      <c r="M73" s="26">
+        <v>1</v>
+      </c>
+      <c r="O73" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P73" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="Q73" s="34">
+      <c r="Q73" s="23">
         <v>82.568531468531461</v>
       </c>
-      <c r="R73" s="38">
+      <c r="R73" s="27">
         <v>7.7031963470319633</v>
       </c>
     </row>
@@ -4804,23 +4871,23 @@
       <c r="J74" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K74" s="17"/>
-      <c r="L74" s="37">
-        <v>2</v>
-      </c>
-      <c r="M74" s="37">
-        <v>2</v>
-      </c>
-      <c r="O74" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P74" s="32" t="s">
+      <c r="K74" s="38"/>
+      <c r="L74" s="26">
+        <v>1</v>
+      </c>
+      <c r="M74" s="26">
+        <v>1</v>
+      </c>
+      <c r="O74" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P74" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="Q74" s="34">
+      <c r="Q74" s="23">
         <v>77.035767935767922</v>
       </c>
-      <c r="R74" s="38">
+      <c r="R74" s="27">
         <v>6.808219178082191</v>
       </c>
     </row>
@@ -4855,23 +4922,23 @@
       <c r="J75" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K75" s="17"/>
-      <c r="L75" s="37">
-        <v>2</v>
-      </c>
-      <c r="M75" s="37">
-        <v>2</v>
-      </c>
-      <c r="O75" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P75" s="32" t="s">
+      <c r="K75" s="38"/>
+      <c r="L75" s="26">
+        <v>1</v>
+      </c>
+      <c r="M75" s="26">
+        <v>1</v>
+      </c>
+      <c r="O75" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P75" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="Q75" s="34">
+      <c r="Q75" s="23">
         <v>77.839186739186729</v>
       </c>
-      <c r="R75" s="38">
+      <c r="R75" s="27">
         <v>7.6514459665144594</v>
       </c>
     </row>
@@ -4906,25 +4973,25 @@
       <c r="J76" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K76" s="17" t="s">
+      <c r="K76" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="L76" s="37">
-        <v>2</v>
-      </c>
-      <c r="M76" s="37">
-        <v>2</v>
-      </c>
-      <c r="O76" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P76" s="32" t="s">
+      <c r="L76" s="26">
+        <v>1</v>
+      </c>
+      <c r="M76" s="26">
+        <v>1</v>
+      </c>
+      <c r="O76" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P76" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="Q76" s="34">
+      <c r="Q76" s="23">
         <v>77.349158249158251</v>
       </c>
-      <c r="R76" s="38">
+      <c r="R76" s="27">
         <v>7.289193302891932</v>
       </c>
     </row>
@@ -4959,23 +5026,23 @@
       <c r="J77" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K77" s="16"/>
-      <c r="L77" s="37">
-        <v>2</v>
-      </c>
-      <c r="M77" s="37">
-        <v>2</v>
-      </c>
-      <c r="O77" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P77" s="32" t="s">
+      <c r="K77" s="11"/>
+      <c r="L77" s="26">
+        <v>1</v>
+      </c>
+      <c r="M77" s="26">
+        <v>1</v>
+      </c>
+      <c r="O77" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P77" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="Q77" s="34">
+      <c r="Q77" s="23">
         <v>76.953146853146848</v>
       </c>
-      <c r="R77" s="38">
+      <c r="R77" s="27">
         <v>6.7336377473363784</v>
       </c>
     </row>
@@ -5010,23 +5077,23 @@
       <c r="J78" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K78" s="16"/>
-      <c r="L78" s="37">
-        <v>2</v>
-      </c>
-      <c r="M78" s="37">
-        <v>2</v>
-      </c>
-      <c r="O78" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P78" s="32" t="s">
+      <c r="K78" s="11"/>
+      <c r="L78" s="26">
+        <v>1</v>
+      </c>
+      <c r="M78" s="26">
+        <v>1</v>
+      </c>
+      <c r="O78" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P78" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="Q78" s="34">
+      <c r="Q78" s="23">
         <v>77.417534317534304</v>
       </c>
-      <c r="R78" s="38">
+      <c r="R78" s="27">
         <v>6.1385083713850825</v>
       </c>
     </row>
@@ -5061,23 +5128,23 @@
       <c r="J79" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K79" s="17"/>
-      <c r="L79" s="37">
-        <v>2</v>
-      </c>
-      <c r="M79" s="37">
-        <v>2</v>
-      </c>
-      <c r="O79" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P79" s="32" t="s">
+      <c r="K79" s="38"/>
+      <c r="L79" s="26">
+        <v>1</v>
+      </c>
+      <c r="M79" s="26">
+        <v>1</v>
+      </c>
+      <c r="O79" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P79" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="Q79" s="34">
+      <c r="Q79" s="23">
         <v>47.599870499870498</v>
       </c>
-      <c r="R79" s="38">
+      <c r="R79" s="27">
         <v>22.278538812785389</v>
       </c>
     </row>
@@ -5112,23 +5179,23 @@
       <c r="J80" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K80" s="17"/>
-      <c r="L80" s="37">
-        <v>2</v>
-      </c>
-      <c r="M80" s="37">
-        <v>2</v>
-      </c>
-      <c r="O80" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P80" s="32" t="s">
+      <c r="K80" s="38"/>
+      <c r="L80" s="26">
+        <v>1</v>
+      </c>
+      <c r="M80" s="26">
+        <v>1</v>
+      </c>
+      <c r="O80" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P80" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="Q80" s="34">
+      <c r="Q80" s="23">
         <v>62.323517223517214</v>
       </c>
-      <c r="R80" s="38">
+      <c r="R80" s="27">
         <v>13.045662100456619</v>
       </c>
     </row>
@@ -5163,23 +5230,23 @@
       <c r="J81" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K81" s="17"/>
-      <c r="L81" s="37">
-        <v>2</v>
-      </c>
-      <c r="M81" s="37">
-        <v>2</v>
-      </c>
-      <c r="O81" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P81" s="32" t="s">
+      <c r="K81" s="38"/>
+      <c r="L81" s="26">
+        <v>1</v>
+      </c>
+      <c r="M81" s="26">
+        <v>1</v>
+      </c>
+      <c r="O81" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P81" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="Q81" s="34">
+      <c r="Q81" s="23">
         <v>74.693887593887595</v>
       </c>
-      <c r="R81" s="38">
+      <c r="R81" s="27">
         <v>5.7260273972602747</v>
       </c>
     </row>
@@ -5214,23 +5281,23 @@
       <c r="J82" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K82" s="17"/>
-      <c r="L82" s="37">
-        <v>2</v>
-      </c>
-      <c r="M82" s="37">
-        <v>2</v>
-      </c>
-      <c r="O82" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P82" s="32" t="s">
+      <c r="K82" s="38"/>
+      <c r="L82" s="26">
+        <v>1</v>
+      </c>
+      <c r="M82" s="26">
+        <v>1</v>
+      </c>
+      <c r="O82" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P82" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="Q82" s="34">
+      <c r="Q82" s="23">
         <v>75.685340585340583</v>
       </c>
-      <c r="R82" s="38">
+      <c r="R82" s="27">
         <v>4.6044140030441403</v>
       </c>
     </row>
@@ -5265,23 +5332,23 @@
       <c r="J83" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K83" s="16"/>
-      <c r="L83" s="37">
-        <v>2</v>
-      </c>
-      <c r="M83" s="37">
-        <v>2</v>
-      </c>
-      <c r="O83" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P83" s="32" t="s">
+      <c r="K83" s="11"/>
+      <c r="L83" s="26">
+        <v>1</v>
+      </c>
+      <c r="M83" s="26">
+        <v>1</v>
+      </c>
+      <c r="O83" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P83" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="Q83" s="34">
+      <c r="Q83" s="23">
         <v>47.739471639471638</v>
       </c>
-      <c r="R83" s="38">
+      <c r="R83" s="27">
         <v>22.312024353120243</v>
       </c>
     </row>
@@ -5316,25 +5383,25 @@
       <c r="J84" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K84" s="16" t="s">
+      <c r="K84" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="L84" s="37">
-        <v>2</v>
-      </c>
-      <c r="M84" s="37">
-        <v>2</v>
-      </c>
-      <c r="O84" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P84" s="32" t="s">
+      <c r="L84" s="26">
+        <v>1</v>
+      </c>
+      <c r="M84" s="26">
+        <v>1</v>
+      </c>
+      <c r="O84" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P84" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="Q84" s="34">
+      <c r="Q84" s="23">
         <v>48.166822066822064</v>
       </c>
-      <c r="R84" s="38">
+      <c r="R84" s="27">
         <v>23.228310502283108</v>
       </c>
     </row>
@@ -5369,23 +5436,23 @@
       <c r="J85" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K85" s="16"/>
-      <c r="L85" s="37">
-        <v>2</v>
-      </c>
-      <c r="M85" s="37">
-        <v>2</v>
-      </c>
-      <c r="O85" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P85" s="32" t="s">
+      <c r="K85" s="11"/>
+      <c r="L85" s="26">
+        <v>1</v>
+      </c>
+      <c r="M85" s="26">
+        <v>1</v>
+      </c>
+      <c r="O85" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P85" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="Q85" s="34">
+      <c r="Q85" s="23">
         <v>61.816394716394711</v>
       </c>
-      <c r="R85" s="38">
+      <c r="R85" s="27">
         <v>14.969558599695588</v>
       </c>
     </row>
@@ -5420,23 +5487,23 @@
       <c r="J86" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K86" s="16"/>
-      <c r="L86" s="37">
-        <v>2</v>
-      </c>
-      <c r="M86" s="37">
-        <v>2</v>
-      </c>
-      <c r="O86" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P86" s="32" t="s">
+      <c r="K86" s="11"/>
+      <c r="L86" s="26">
+        <v>1</v>
+      </c>
+      <c r="M86" s="26">
+        <v>1</v>
+      </c>
+      <c r="O86" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P86" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="Q86" s="34">
+      <c r="Q86" s="23">
         <v>74.756565656565641</v>
       </c>
-      <c r="R86" s="38">
+      <c r="R86" s="27">
         <v>4.6304414003044139</v>
       </c>
     </row>
@@ -5471,23 +5538,23 @@
       <c r="J87" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K87" s="16"/>
-      <c r="L87" s="37">
-        <v>2</v>
-      </c>
-      <c r="M87" s="37">
-        <v>2</v>
-      </c>
-      <c r="O87" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P87" s="32" t="s">
+      <c r="K87" s="11"/>
+      <c r="L87" s="26">
+        <v>1</v>
+      </c>
+      <c r="M87" s="26">
+        <v>1</v>
+      </c>
+      <c r="O87" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P87" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="Q87" s="34">
+      <c r="Q87" s="23">
         <v>76.423232323232313</v>
       </c>
-      <c r="R87" s="38">
+      <c r="R87" s="27">
         <v>4.7433789954337895</v>
       </c>
     </row>
@@ -5522,25 +5589,25 @@
       <c r="J88" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K88" s="17" t="s">
+      <c r="K88" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="L88" s="37">
-        <v>2</v>
-      </c>
-      <c r="M88" s="37">
-        <v>2</v>
-      </c>
-      <c r="O88" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P88" s="32" t="s">
+      <c r="L88" s="26">
+        <v>1</v>
+      </c>
+      <c r="M88" s="26">
+        <v>1</v>
+      </c>
+      <c r="O88" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P88" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="Q88" s="34">
+      <c r="Q88" s="23">
         <v>71.394742294742287</v>
       </c>
-      <c r="R88" s="38">
+      <c r="R88" s="27">
         <v>12.137499999999999</v>
       </c>
     </row>
@@ -5575,23 +5642,23 @@
       <c r="J89" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K89" s="17"/>
-      <c r="L89" s="37">
-        <v>2</v>
-      </c>
-      <c r="M89" s="37">
-        <v>2</v>
-      </c>
-      <c r="O89" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P89" s="32" t="s">
+      <c r="K89" s="38"/>
+      <c r="L89" s="26">
+        <v>1</v>
+      </c>
+      <c r="M89" s="26">
+        <v>1</v>
+      </c>
+      <c r="O89" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P89" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="Q89" s="34">
+      <c r="Q89" s="23">
         <v>73.836337736337725</v>
       </c>
-      <c r="R89" s="38">
+      <c r="R89" s="27">
         <v>5.3083333333333336</v>
       </c>
     </row>
@@ -5626,23 +5693,23 @@
       <c r="J90" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K90" s="17"/>
-      <c r="L90" s="37">
-        <v>2</v>
-      </c>
-      <c r="M90" s="37">
-        <v>2</v>
-      </c>
-      <c r="O90" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P90" s="32" t="s">
+      <c r="K90" s="38"/>
+      <c r="L90" s="26">
+        <v>1</v>
+      </c>
+      <c r="M90" s="26">
+        <v>1</v>
+      </c>
+      <c r="O90" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P90" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="Q90" s="34">
+      <c r="Q90" s="23">
         <v>75.654001554001539</v>
       </c>
-      <c r="R90" s="38">
+      <c r="R90" s="27">
         <v>5.4208333333333334</v>
       </c>
     </row>
@@ -5677,23 +5744,23 @@
       <c r="J91" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K91" s="16"/>
-      <c r="L91" s="37">
-        <v>2</v>
-      </c>
-      <c r="M91" s="37">
-        <v>2</v>
-      </c>
-      <c r="O91" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P91" s="32" t="s">
+      <c r="K91" s="11"/>
+      <c r="L91" s="26">
+        <v>1</v>
+      </c>
+      <c r="M91" s="26">
+        <v>1</v>
+      </c>
+      <c r="O91" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P91" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="Q91" s="34">
+      <c r="Q91" s="23">
         <v>49.793602693602679</v>
       </c>
-      <c r="R91" s="38">
+      <c r="R91" s="27">
         <v>20.140277777777779</v>
       </c>
     </row>
@@ -5728,23 +5795,23 @@
       <c r="J92" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K92" s="16"/>
-      <c r="L92" s="37">
-        <v>2</v>
-      </c>
-      <c r="M92" s="37">
-        <v>2</v>
-      </c>
-      <c r="O92" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P92" s="32" t="s">
+      <c r="K92" s="11"/>
+      <c r="L92" s="26">
+        <v>1</v>
+      </c>
+      <c r="M92" s="26">
+        <v>1</v>
+      </c>
+      <c r="O92" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P92" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="Q92" s="34">
+      <c r="Q92" s="23">
         <v>64.651152551152549</v>
       </c>
-      <c r="R92" s="38">
+      <c r="R92" s="27">
         <v>12.384722222222223</v>
       </c>
     </row>
@@ -5779,23 +5846,23 @@
       <c r="J93" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K93" s="16"/>
-      <c r="L93" s="37">
-        <v>2</v>
-      </c>
-      <c r="M93" s="37">
-        <v>2</v>
-      </c>
-      <c r="O93" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P93" s="32" t="s">
+      <c r="K93" s="11"/>
+      <c r="L93" s="26">
+        <v>1</v>
+      </c>
+      <c r="M93" s="26">
+        <v>1</v>
+      </c>
+      <c r="O93" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P93" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="Q93" s="34">
+      <c r="Q93" s="23">
         <v>74.275084175084174</v>
       </c>
-      <c r="R93" s="38">
+      <c r="R93" s="27">
         <v>4.6138888888888889</v>
       </c>
     </row>
@@ -5830,25 +5897,25 @@
       <c r="J94" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K94" s="16" t="s">
+      <c r="K94" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="L94" s="37">
-        <v>2</v>
-      </c>
-      <c r="M94" s="37">
-        <v>2</v>
-      </c>
-      <c r="O94" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P94" s="32" t="s">
+      <c r="L94" s="26">
+        <v>1</v>
+      </c>
+      <c r="M94" s="26">
+        <v>1</v>
+      </c>
+      <c r="O94" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P94" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="Q94" s="34">
+      <c r="Q94" s="23">
         <v>73.571380471380465</v>
       </c>
-      <c r="R94" s="38">
+      <c r="R94" s="27">
         <v>4.8305555555555557</v>
       </c>
     </row>
@@ -5883,23 +5950,23 @@
       <c r="J95" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K95" s="16"/>
-      <c r="L95" s="37">
-        <v>2</v>
-      </c>
-      <c r="M95" s="37">
-        <v>2</v>
-      </c>
-      <c r="O95" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P95" s="32" t="s">
+      <c r="K95" s="11"/>
+      <c r="L95" s="26">
+        <v>1</v>
+      </c>
+      <c r="M95" s="26">
+        <v>1</v>
+      </c>
+      <c r="O95" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P95" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="Q95" s="34">
+      <c r="Q95" s="23">
         <v>76.830639730639732</v>
       </c>
-      <c r="R95" s="38">
+      <c r="R95" s="27">
         <v>4.3402777777777786</v>
       </c>
     </row>
@@ -5934,23 +6001,23 @@
       <c r="J96" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K96" s="17"/>
-      <c r="L96" s="37">
-        <v>2</v>
-      </c>
-      <c r="M96" s="37">
-        <v>2</v>
-      </c>
-      <c r="O96" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P96" s="32" t="s">
+      <c r="K96" s="38"/>
+      <c r="L96" s="26">
+        <v>1</v>
+      </c>
+      <c r="M96" s="26">
+        <v>1</v>
+      </c>
+      <c r="O96" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P96" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="Q96" s="34">
+      <c r="Q96" s="23">
         <v>65.890468790468788</v>
       </c>
-      <c r="R96" s="38">
+      <c r="R96" s="27">
         <v>12.212499999999999</v>
       </c>
     </row>
@@ -5985,23 +6052,23 @@
       <c r="J97" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K97" s="17"/>
-      <c r="L97" s="37">
-        <v>2</v>
-      </c>
-      <c r="M97" s="37">
-        <v>2</v>
-      </c>
-      <c r="O97" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P97" s="32" t="s">
+      <c r="K97" s="38"/>
+      <c r="L97" s="26">
+        <v>1</v>
+      </c>
+      <c r="M97" s="26">
+        <v>1</v>
+      </c>
+      <c r="O97" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P97" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="Q97" s="34">
+      <c r="Q97" s="23">
         <v>76.30642320642319</v>
       </c>
-      <c r="R97" s="38">
+      <c r="R97" s="27">
         <v>4.5283333333333333</v>
       </c>
     </row>
@@ -6036,23 +6103,23 @@
       <c r="J98" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K98" s="17"/>
-      <c r="L98" s="37">
-        <v>2</v>
-      </c>
-      <c r="M98" s="37">
-        <v>2</v>
-      </c>
-      <c r="O98" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P98" s="32" t="s">
+      <c r="K98" s="38"/>
+      <c r="L98" s="26">
+        <v>1</v>
+      </c>
+      <c r="M98" s="26">
+        <v>1</v>
+      </c>
+      <c r="O98" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P98" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="Q98" s="34">
+      <c r="Q98" s="23">
         <v>74.312121212121198</v>
       </c>
-      <c r="R98" s="38">
+      <c r="R98" s="27">
         <v>3.8968055555555563</v>
       </c>
     </row>
@@ -6087,23 +6154,23 @@
       <c r="J99" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K99" s="16"/>
-      <c r="L99" s="37">
-        <v>2</v>
-      </c>
-      <c r="M99" s="37">
-        <v>2</v>
-      </c>
-      <c r="O99" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P99" s="32" t="s">
+      <c r="K99" s="11"/>
+      <c r="L99" s="26">
+        <v>1</v>
+      </c>
+      <c r="M99" s="26">
+        <v>1</v>
+      </c>
+      <c r="O99" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P99" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="Q99" s="34">
+      <c r="Q99" s="23">
         <v>66.317819217819221</v>
       </c>
-      <c r="R99" s="38">
+      <c r="R99" s="27">
         <v>12.647222222222226</v>
       </c>
     </row>
@@ -6138,23 +6205,23 @@
       <c r="J100" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K100" s="16"/>
-      <c r="L100" s="37">
-        <v>2</v>
-      </c>
-      <c r="M100" s="37">
-        <v>2</v>
-      </c>
-      <c r="O100" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P100" s="32" t="s">
+      <c r="K100" s="11"/>
+      <c r="L100" s="26">
+        <v>1</v>
+      </c>
+      <c r="M100" s="26">
+        <v>1</v>
+      </c>
+      <c r="O100" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P100" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="Q100" s="34">
+      <c r="Q100" s="23">
         <v>77.765112665112667</v>
       </c>
-      <c r="R100" s="38">
+      <c r="R100" s="27">
         <v>4.7333333333333334</v>
       </c>
     </row>
@@ -6189,23 +6256,23 @@
       <c r="J101" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K101" s="16"/>
-      <c r="L101" s="37">
-        <v>2</v>
-      </c>
-      <c r="M101" s="37">
-        <v>2</v>
-      </c>
-      <c r="O101" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P101" s="32" t="s">
+      <c r="K101" s="11"/>
+      <c r="L101" s="26">
+        <v>1</v>
+      </c>
+      <c r="M101" s="26">
+        <v>1</v>
+      </c>
+      <c r="O101" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P101" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="Q101" s="34">
+      <c r="Q101" s="23">
         <v>77.591323491323493</v>
       </c>
-      <c r="R101" s="38">
+      <c r="R101" s="27">
         <v>4.8263888888888893</v>
       </c>
     </row>
@@ -6240,23 +6307,23 @@
       <c r="J102" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K102" s="17"/>
-      <c r="L102" s="37">
-        <v>2</v>
-      </c>
-      <c r="M102" s="37">
-        <v>2</v>
-      </c>
-      <c r="O102" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P102" s="32" t="s">
+      <c r="K102" s="38"/>
+      <c r="L102" s="26">
+        <v>1</v>
+      </c>
+      <c r="M102" s="26">
+        <v>1</v>
+      </c>
+      <c r="O102" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P102" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="Q102" s="34">
+      <c r="Q102" s="23">
         <v>77.651152551152549</v>
       </c>
-      <c r="R102" s="38">
+      <c r="R102" s="27">
         <v>4.7944444444444452</v>
       </c>
     </row>
@@ -6291,27 +6358,27 @@
       <c r="J103" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K103" s="17"/>
-      <c r="L103" s="37">
-        <v>2</v>
-      </c>
-      <c r="M103" s="37">
-        <v>2</v>
-      </c>
-      <c r="O103" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P103" s="32" t="s">
+      <c r="K103" s="38"/>
+      <c r="L103" s="26">
+        <v>1</v>
+      </c>
+      <c r="M103" s="26">
+        <v>1</v>
+      </c>
+      <c r="O103" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P103" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="Q103" s="34">
+      <c r="Q103" s="23">
         <v>77.80499870499871</v>
       </c>
-      <c r="R103" s="38">
+      <c r="R103" s="27">
         <v>4.4577777777777783</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="57.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>27</v>
       </c>
@@ -6345,22 +6412,22 @@
       <c r="K104" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="L104" s="37">
-        <v>2</v>
-      </c>
-      <c r="M104" s="37">
-        <v>2</v>
-      </c>
-      <c r="O104" s="36">
-        <v>46134</v>
-      </c>
-      <c r="P104" s="32" t="s">
+      <c r="L104" s="26">
+        <v>1</v>
+      </c>
+      <c r="M104" s="26">
+        <v>1</v>
+      </c>
+      <c r="O104" s="25">
+        <v>46134</v>
+      </c>
+      <c r="P104" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="Q104" s="34">
+      <c r="Q104" s="23">
         <v>92.198161098161108</v>
       </c>
-      <c r="R104" s="38">
+      <c r="R104" s="27">
         <v>9.9222222222222207</v>
       </c>
     </row>
@@ -6375,7 +6442,7 @@
       <c r="H105" s="10"/>
       <c r="I105" s="10"/>
       <c r="J105" s="9"/>
-      <c r="K105" s="20"/>
+      <c r="K105" s="40"/>
     </row>
     <row r="106" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A106" s="9"/>
@@ -6388,7 +6455,7 @@
       <c r="H106" s="10"/>
       <c r="I106" s="10"/>
       <c r="J106" s="9"/>
-      <c r="K106" s="20"/>
+      <c r="K106" s="40"/>
     </row>
     <row r="107" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A107" s="9"/>
@@ -6401,7 +6468,7 @@
       <c r="H107" s="10"/>
       <c r="I107" s="10"/>
       <c r="J107" s="9"/>
-      <c r="K107" s="20"/>
+      <c r="K107" s="40"/>
     </row>
     <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A108" s="9"/>
@@ -6414,7 +6481,7 @@
       <c r="H108" s="9"/>
       <c r="I108" s="9"/>
       <c r="J108" s="9"/>
-      <c r="K108" s="20"/>
+      <c r="K108" s="40"/>
     </row>
     <row r="109" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A109" s="9"/>
@@ -6427,7 +6494,7 @@
       <c r="H109" s="9"/>
       <c r="I109" s="9"/>
       <c r="J109" s="9"/>
-      <c r="K109" s="20"/>
+      <c r="K109" s="40"/>
     </row>
     <row r="110" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A110" s="9"/>
@@ -6440,7 +6507,7 @@
       <c r="H110" s="9"/>
       <c r="I110" s="9"/>
       <c r="J110" s="9"/>
-      <c r="K110" s="20"/>
+      <c r="K110" s="40"/>
     </row>
     <row r="111" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A111" s="9"/>
@@ -6453,7 +6520,7 @@
       <c r="H111" s="9"/>
       <c r="I111" s="9"/>
       <c r="J111" s="9"/>
-      <c r="K111" s="20"/>
+      <c r="K111" s="40"/>
     </row>
     <row r="112" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A112" s="9"/>
@@ -6466,7 +6533,7 @@
       <c r="H112" s="9"/>
       <c r="I112" s="9"/>
       <c r="J112" s="9"/>
-      <c r="K112" s="20"/>
+      <c r="K112" s="40"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="9"/>
@@ -6479,7 +6546,7 @@
       <c r="H113" s="9"/>
       <c r="I113" s="9"/>
       <c r="J113" s="9"/>
-      <c r="K113" s="20"/>
+      <c r="K113" s="40"/>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="9"/>
@@ -6492,7 +6559,7 @@
       <c r="H114" s="9"/>
       <c r="I114" s="9"/>
       <c r="J114" s="9"/>
-      <c r="K114" s="20"/>
+      <c r="K114" s="40"/>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="9"/>
@@ -6505,7 +6572,7 @@
       <c r="H115" s="9"/>
       <c r="I115" s="9"/>
       <c r="J115" s="9"/>
-      <c r="K115" s="20"/>
+      <c r="K115" s="40"/>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="9"/>
@@ -6518,7 +6585,7 @@
       <c r="H116" s="9"/>
       <c r="I116" s="9"/>
       <c r="J116" s="9"/>
-      <c r="K116" s="20"/>
+      <c r="K116" s="40"/>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="9"/>
@@ -6531,7 +6598,7 @@
       <c r="H117" s="9"/>
       <c r="I117" s="9"/>
       <c r="J117" s="9"/>
-      <c r="K117" s="20"/>
+      <c r="K117" s="40"/>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="9"/>
@@ -6544,7 +6611,7 @@
       <c r="H118" s="9"/>
       <c r="I118" s="9"/>
       <c r="J118" s="9"/>
-      <c r="K118" s="20"/>
+      <c r="K118" s="40"/>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="9"/>
@@ -6557,7 +6624,7 @@
       <c r="H119" s="9"/>
       <c r="I119" s="9"/>
       <c r="J119" s="9"/>
-      <c r="K119" s="20"/>
+      <c r="K119" s="40"/>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="9"/>
@@ -6570,7 +6637,7 @@
       <c r="H120" s="9"/>
       <c r="I120" s="9"/>
       <c r="J120" s="9"/>
-      <c r="K120" s="20"/>
+      <c r="K120" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.25" header="0.3" footer="0.3"/>
@@ -6579,20 +6646,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e362b6aa-9e52-454d-a744-a011f894490f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e362b6aa-9e52-454d-a744-a011f894490f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6778,6 +6845,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C56E6CDE-B1D8-4B8C-A235-CFA6F399302F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EBAD766-690B-4B4D-8BA3-45BBCD0E4195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -6789,14 +6864,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="e362b6aa-9e52-454d-a744-a011f894490f"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C56E6CDE-B1D8-4B8C-A235-CFA6F399302F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>